<commit_message>
Update documents with COM71 codes change
Codes updated to Y, N, TYPE I, TYPE II, TYPE UNKNOWN, TYPE OTHER.
'TYPE I' and 'TYPE II' restored to match the V4 codes, correcting the typo introduced in V5 as 'TYPE1' and 'TYPE2'.
</commit_message>
<xml_diff>
--- a/Excel/v5/UKRR DataSet Amendments.xlsx
+++ b/Excel/v5/UKRR DataSet Amendments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marta.badji\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1A85E5-D4D3-4926-A034-C669B2A91B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4F8BAAAB-3E82-4785-A9C2-B1C93A0C366B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,11 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Amendments!$C$1:$J$3</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -36,364 +39,388 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="132">
-  <si>
-    <t>Format</t>
-  </si>
-  <si>
-    <t>Item Description</t>
-  </si>
-  <si>
-    <t>CODES / CODELISTS</t>
-  </si>
-  <si>
-    <t>Unit of Measurement</t>
-  </si>
-  <si>
-    <t>IF / Qualification</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>N4</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>DXS01</t>
-  </si>
-  <si>
-    <t>EDTA primary renal disease code</t>
-  </si>
-  <si>
-    <t>https://era-edta-reg.org/prd.jsp?disclaim=1</t>
-  </si>
-  <si>
-    <t>Previously ERFAJ.  All patients with eGFR&lt;30 and on RRT</t>
-  </si>
-  <si>
-    <t>Diagnoses/RenalDiagnosis</t>
-  </si>
-  <si>
-    <t>DXS02</t>
-  </si>
-  <si>
-    <t>SNOMED primary renal disease code</t>
-  </si>
-  <si>
-    <t>Please contact UKRR for constrained list</t>
-  </si>
-  <si>
-    <t>DXS03</t>
-  </si>
-  <si>
-    <t>Y, N, UNKNOWN</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/valueset-example-yesnodontknow.html  and http://hl7.org/fhir/codesystem-data-absent-reason.html#data-absent-reason-asked-unknown</t>
-  </si>
-  <si>
-    <t>DXS04</t>
-  </si>
-  <si>
-    <t>Secondary renal disease code</t>
-  </si>
-  <si>
-    <t>Previously ERF07</t>
-  </si>
-  <si>
-    <t>DXS05</t>
-  </si>
-  <si>
-    <t>Primary disease free text if no suitable code available</t>
-  </si>
-  <si>
-    <t>DXS06</t>
-  </si>
-  <si>
-    <t>Date of diagnosis of primary renal disease</t>
-  </si>
-  <si>
-    <t>DXS07</t>
-  </si>
-  <si>
-    <t>Diabetes</t>
-  </si>
-  <si>
-    <t>N, TYPE1, TYPE2, TYPE UNKNOWN</t>
-  </si>
-  <si>
-    <t>Diagnoses/Diagnosis</t>
-  </si>
-  <si>
-    <t>DXS08</t>
-  </si>
-  <si>
-    <t>Date diabetes diagnosed</t>
-  </si>
-  <si>
-    <t>Required if DXS07 not N or blank</t>
-  </si>
-  <si>
-    <t>DXS09</t>
-  </si>
-  <si>
-    <t>Malignancy Yes / No</t>
-  </si>
-  <si>
-    <t>If Yes there should be a code in DXS10 and a date in DXS11</t>
-  </si>
-  <si>
-    <t>DXS10</t>
-  </si>
-  <si>
-    <t>Malignancy site, first primary site only</t>
-  </si>
-  <si>
-    <t>Codelist RR19</t>
-  </si>
-  <si>
-    <t>DXS11</t>
-  </si>
-  <si>
-    <t>Malignancy  - date first diagnosed</t>
-  </si>
-  <si>
-    <t>N1</t>
-  </si>
-  <si>
-    <t>N3</t>
-  </si>
-  <si>
-    <t>nnn.n</t>
-  </si>
-  <si>
-    <t>Observations/Observation</t>
-  </si>
-  <si>
-    <t>LabOrders/LabOrder/ResultItems</t>
-  </si>
-  <si>
-    <t>nn.n</t>
-  </si>
-  <si>
-    <t>Glomerular filtration rate (GFR) predicted by creatinine based formula (CKD-EPI) WITHOUT ethnicity</t>
-  </si>
-  <si>
-    <t>N2</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>QBLE5</t>
-  </si>
-  <si>
-    <t>White blood count (WBC)</t>
-  </si>
-  <si>
-    <t>QBLE4</t>
-  </si>
-  <si>
-    <t>Platelets</t>
-  </si>
-  <si>
-    <t>QBLJJ</t>
-  </si>
-  <si>
-    <t>QBLF3</t>
-  </si>
-  <si>
-    <t>QBLC1</t>
-  </si>
-  <si>
-    <t>nnnnn.n</t>
-  </si>
-  <si>
-    <t>Urine protein:creatinine ratio</t>
-  </si>
-  <si>
-    <t>QBLC3</t>
-  </si>
-  <si>
-    <t>nnnn.n</t>
-  </si>
-  <si>
-    <t>Urine albumin:creatinine ratio</t>
-  </si>
-  <si>
-    <t>QBLJN</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>&gt;100, 70, 30, &lt;5</t>
-  </si>
-  <si>
-    <t>RR1 - Hospital Sites</t>
-  </si>
-  <si>
-    <t>RR2 - Access Type</t>
-  </si>
-  <si>
-    <t>RR22 - Medication Route</t>
-  </si>
-  <si>
-    <t>RR23 - Medication Units</t>
-  </si>
-  <si>
-    <t>pg</t>
-  </si>
-  <si>
-    <t>Either DXS01 or DXS02 is required</t>
-  </si>
-  <si>
-    <t>Previously ERF09. Additional text to describe PRD when neither EDTA nor SNOMED code is available</t>
-  </si>
-  <si>
-    <t>Was primary renal disease diagnosis confirmed by kidney biopsy?</t>
-  </si>
-  <si>
-    <t>Valid only if PD</t>
-  </si>
-  <si>
-    <t>Reticulocyte haemoglobin (CHr)</t>
-  </si>
-  <si>
-    <t>PD fluid WCC count</t>
-  </si>
-  <si>
-    <t>Glomerular filtration rate (GFR) predicted by creatinine based formula (MDRD) WITHOUT ethnicity</t>
-  </si>
-  <si>
-    <t>QBLAP</t>
-  </si>
-  <si>
-    <t>QBLAR</t>
-  </si>
-  <si>
-    <t>UKRDC / RDA Mapping</t>
-  </si>
-  <si>
-    <t>mL/min/1.72m^2</t>
-  </si>
-  <si>
-    <t>10^9/L</t>
-  </si>
-  <si>
-    <t>mg/mmol</t>
-  </si>
-  <si>
-    <t>SNOMED</t>
-  </si>
-  <si>
-    <t>ERFAJ</t>
-  </si>
-  <si>
-    <t>ERF07</t>
-  </si>
-  <si>
-    <t>ERF09</t>
-  </si>
-  <si>
-    <t>Additional text to describe PRD when neither EDTA nor SNOMED code is available</t>
-  </si>
-  <si>
-    <t>All patients with eGFR&lt;30 and on RRT</t>
-  </si>
-  <si>
-    <t>COM71</t>
-  </si>
-  <si>
-    <t>COM72</t>
-  </si>
-  <si>
-    <t>COM81</t>
-  </si>
-  <si>
-    <t>COM82</t>
-  </si>
-  <si>
-    <t>COM83</t>
-  </si>
-  <si>
-    <t>Required if COM71 not N or blank</t>
-  </si>
-  <si>
-    <t>If Yes there should be a code in COM82 and a date in COM83</t>
-  </si>
-  <si>
-    <t>ERFAK</t>
-  </si>
-  <si>
-    <t>ERF92</t>
-  </si>
-  <si>
-    <t>ERF93</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="135">
   <si>
     <t>Amendments</t>
+  </si>
+  <si>
+    <t>Effective in version</t>
+  </si>
+  <si>
+    <t>Amendment</t>
   </si>
   <si>
     <t>Field ID/
 Item name</t>
   </si>
   <si>
+    <t>Coding standard</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>Item Description</t>
+  </si>
+  <si>
+    <t>CODES / CODELISTS</t>
+  </si>
+  <si>
+    <t>Unit of Measurement</t>
+  </si>
+  <si>
+    <t>IF / Qualification</t>
+  </si>
+  <si>
+    <t>UKRDC / RDA Mapping</t>
+  </si>
+  <si>
     <t>Comments</t>
   </si>
   <si>
-    <t>Amendment</t>
-  </si>
-  <si>
     <t>Removed</t>
   </si>
   <si>
+    <t>DXS01</t>
+  </si>
+  <si>
+    <t>N4</t>
+  </si>
+  <si>
+    <t>EDTA primary renal disease code</t>
+  </si>
+  <si>
+    <t>https://era-edta-reg.org/prd.jsp?disclaim=1</t>
+  </si>
+  <si>
+    <t>Previously ERFAJ.  All patients with eGFR&lt;30 and on RRT</t>
+  </si>
+  <si>
+    <t>Diagnoses/RenalDiagnosis</t>
+  </si>
+  <si>
+    <t>DXS (Diagnoses) block removed, items moved to the ERF (Renal diagnoses) and COM (Comorbidities) blocks</t>
+  </si>
+  <si>
+    <t>DXS02</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>SNOMED primary renal disease code</t>
+  </si>
+  <si>
+    <t>Please contact UKRR for constrained list</t>
+  </si>
+  <si>
+    <t>Either DXS01 or DXS02 is required</t>
+  </si>
+  <si>
+    <t>DXS03</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Was primary renal disease diagnosis confirmed by kidney biopsy?</t>
+  </si>
+  <si>
+    <t>Y, N, UNKNOWN</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/valueset-example-yesnodontknow.html  and http://hl7.org/fhir/codesystem-data-absent-reason.html#data-absent-reason-asked-unknown</t>
+  </si>
+  <si>
+    <t>DXS04</t>
+  </si>
+  <si>
+    <t>Secondary renal disease code</t>
+  </si>
+  <si>
+    <t>Previously ERF07</t>
+  </si>
+  <si>
+    <t>DXS05</t>
+  </si>
+  <si>
+    <t>Primary disease free text if no suitable code available</t>
+  </si>
+  <si>
+    <t>Previously ERF09. Additional text to describe PRD when neither EDTA nor SNOMED code is available</t>
+  </si>
+  <si>
+    <t>DXS06</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Date of diagnosis of primary renal disease</t>
+  </si>
+  <si>
+    <t>DXS07</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
+    <t>N, TYPE1, TYPE2, TYPE UNKNOWN</t>
+  </si>
+  <si>
+    <t>Diagnoses/Diagnosis</t>
+  </si>
+  <si>
+    <t>DXS08</t>
+  </si>
+  <si>
+    <t>Date diabetes diagnosed</t>
+  </si>
+  <si>
+    <t>Required if DXS07 not N or blank</t>
+  </si>
+  <si>
+    <t>DXS09</t>
+  </si>
+  <si>
+    <t>Malignancy Yes / No</t>
+  </si>
+  <si>
+    <t>If Yes there should be a code in DXS10 and a date in DXS11</t>
+  </si>
+  <si>
+    <t>DXS10</t>
+  </si>
+  <si>
+    <t>Malignancy site, first primary site only</t>
+  </si>
+  <si>
+    <t>Codelist RR19</t>
+  </si>
+  <si>
+    <t>DXS11</t>
+  </si>
+  <si>
+    <t>Malignancy  - date first diagnosed</t>
+  </si>
+  <si>
     <t>Reinstated</t>
   </si>
   <si>
+    <t>ERFAJ</t>
+  </si>
+  <si>
+    <t>All patients with eGFR&lt;30 and on RRT</t>
+  </si>
+  <si>
+    <t>These items replace DXS01 - DXS06 items.</t>
+  </si>
+  <si>
     <t>Added</t>
   </si>
   <si>
-    <t>DXS (Diagnoses) block removed, items moved to the ERF (Renal diagnoses) and COM (Comorbidities) blocks</t>
-  </si>
-  <si>
-    <t>These items replace DXS01 - DXS06 items.</t>
-  </si>
-  <si>
-    <t>These items replace DXS07 - DXS011 items.</t>
-  </si>
-  <si>
-    <t>Coding standard</t>
+    <t>ERFAK</t>
+  </si>
+  <si>
+    <t>ERF92</t>
+  </si>
+  <si>
+    <t>ERF07</t>
+  </si>
+  <si>
+    <t>ERF09</t>
+  </si>
+  <si>
+    <t>Additional text to describe PRD when neither EDTA nor SNOMED code is available</t>
+  </si>
+  <si>
+    <t>ERF93</t>
+  </si>
+  <si>
+    <t>COM71</t>
+  </si>
+  <si>
+    <t>COM72</t>
+  </si>
+  <si>
+    <t>Required if COM71 not N or blank</t>
+  </si>
+  <si>
+    <t>COM81</t>
+  </si>
+  <si>
+    <t>If Yes there should be a code in COM82 and a date in COM83</t>
+  </si>
+  <si>
+    <t>COM82</t>
+  </si>
+  <si>
+    <t>COM83</t>
+  </si>
+  <si>
+    <t>SNOMED</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>Canadian Study of Health and Aging Clinical Frailty Scale score (Rockwell score)</t>
+  </si>
+  <si>
+    <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+  </si>
+  <si>
+    <t>Observations/Observation</t>
+  </si>
+  <si>
+    <t>QBLF3</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>Transferrin saturation percentage</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>LabOrders/LabOrder/ResultItems</t>
+  </si>
+  <si>
+    <t>Item description changed from 'Transferrin saturation' to 'Transferrin saturation percentage'</t>
+  </si>
+  <si>
+    <t>QBLAP</t>
+  </si>
+  <si>
+    <t>N3</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate (GFR) predicted by creatinine based formula (CKD-EPI) WITHOUT ethnicity</t>
+  </si>
+  <si>
+    <t>mL/min/1.72m^2</t>
+  </si>
+  <si>
+    <t>Unit of measure added</t>
+  </si>
+  <si>
+    <t>QBLAR</t>
+  </si>
+  <si>
+    <t>Glomerular filtration rate (GFR) predicted by creatinine based formula (MDRD) WITHOUT ethnicity</t>
+  </si>
+  <si>
+    <t>QBLE5</t>
+  </si>
+  <si>
+    <t>nnn.n</t>
+  </si>
+  <si>
+    <t>White blood count (WBC)</t>
+  </si>
+  <si>
+    <t>10^9/L</t>
+  </si>
+  <si>
+    <t>QBLE4</t>
+  </si>
+  <si>
+    <t>Platelets</t>
+  </si>
+  <si>
+    <t>QBLJJ</t>
+  </si>
+  <si>
+    <t>nn.n</t>
+  </si>
+  <si>
+    <t>Reticulocyte haemoglobin (CHr)</t>
+  </si>
+  <si>
+    <t>pg</t>
+  </si>
+  <si>
+    <t>QBLC1</t>
+  </si>
+  <si>
+    <t>nnnnn.n</t>
+  </si>
+  <si>
+    <t>Urine protein:creatinine ratio</t>
+  </si>
+  <si>
+    <t>mg/mmol</t>
+  </si>
+  <si>
+    <t>QBLC3</t>
+  </si>
+  <si>
+    <t>nnnn.n</t>
+  </si>
+  <si>
+    <t>Urine albumin:creatinine ratio</t>
+  </si>
+  <si>
+    <t>QBLJN</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>PD fluid WCC count</t>
+  </si>
+  <si>
+    <t>&gt;100, 70, 30, &lt;5</t>
+  </si>
+  <si>
+    <t>cells/uL</t>
+  </si>
+  <si>
+    <t>Valid only if PD</t>
   </si>
   <si>
     <t>Amended codelist</t>
   </si>
   <si>
+    <t>RR1 - Hospital Sites</t>
+  </si>
+  <si>
+    <t>Added RAJ Mid-South Essex and 995 UNKNOWN</t>
+  </si>
+  <si>
+    <t>RR2 - Access Type</t>
+  </si>
+  <si>
     <t>Added UNK Unknown</t>
   </si>
   <si>
+    <t>RR22 - Medication Route</t>
+  </si>
+  <si>
     <t>Added 6 Rectal</t>
   </si>
   <si>
+    <t>RR23 - Medication Units</t>
+  </si>
+  <si>
     <t>Added ug micrograms</t>
   </si>
   <si>
-    <t>cells/uL</t>
-  </si>
-  <si>
-    <t>Transferrin saturation percentage</t>
-  </si>
-  <si>
-    <t>Canadian Study of Health and Aging Clinical Frailty Scale score (Rockwell score)</t>
-  </si>
-  <si>
-    <t>Added RAJ Mid-South Essex and 995 UNKNOWN</t>
+    <t>Tab removed</t>
+  </si>
+  <si>
+    <t>PV data items</t>
+  </si>
+  <si>
+    <t>Ranges removed</t>
+  </si>
+  <si>
+    <t>Lab Results</t>
+  </si>
+  <si>
+    <t>Observations</t>
   </si>
   <si>
     <t>New data items</t>
@@ -405,34 +432,20 @@
     <t>Removed items</t>
   </si>
   <si>
-    <t>Item updated</t>
-  </si>
-  <si>
-    <t>Item description changed from 'Transferrin saturation' to 'Transferrin saturation percentage'</t>
-  </si>
-  <si>
-    <t>Unit of measure added</t>
-  </si>
-  <si>
-    <t>Effective in version</t>
-  </si>
-  <si>
-    <t>Tab removed</t>
-  </si>
-  <si>
-    <t>PV data items</t>
-  </si>
-  <si>
-    <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-  </si>
-  <si>
-    <t>Ranges removed</t>
-  </si>
-  <si>
-    <t>Observations</t>
-  </si>
-  <si>
-    <t>Lab Results</t>
+    <t>Updated</t>
+  </si>
+  <si>
+    <t>Reinstated and updated</t>
+  </si>
+  <si>
+    <t>Y, N, TYPE I, TYPE II, TYPE UNKNOWN, TYPE OTHER</t>
+  </si>
+  <si>
+    <t>These items replace DXS08 - DXS011 items.</t>
+  </si>
+  <si>
+    <t>This item replaces DXS07.
+Codes updated from the V5 values (N, TYPE1, TYPE2, TYPE UNKNOWN). 'TYPE I' and 'TYPE II' restored to match the V4 codes, correcting the typo introduced in V5 as 'TYPE1' and 'TYPE2'.</t>
   </si>
 </sst>
 </file>
@@ -558,7 +571,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -618,6 +631,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -625,7 +653,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -759,6 +787,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1156,9 +1193,9 @@
   <dimension ref="A1:K46"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.1640625" customWidth="1"/>
-    <col min="3" max="3" width="21.6640625" customWidth="1"/>
-    <col min="4" max="4" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="17.08203125" customWidth="1"/>
+    <col min="3" max="3" width="21.58203125" customWidth="1"/>
+    <col min="4" max="4" width="13.08203125" customWidth="1"/>
     <col min="5" max="5" width="9.5" customWidth="1"/>
     <col min="6" max="6" width="46.58203125" customWidth="1"/>
     <col min="7" max="7" width="41.58203125" customWidth="1"/>
@@ -1171,42 +1208,42 @@
   <sheetData>
     <row r="1" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="47" t="s">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>101</v>
+        <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>110</v>
+        <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>102</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
@@ -1214,30 +1251,30 @@
         <v>5.2</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="27" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G4" s="29" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H4" s="30"/>
       <c r="I4" s="28" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="J4" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K4" s="48" t="s">
-        <v>107</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -1245,27 +1282,27 @@
         <v>5.2</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D5" s="27"/>
       <c r="E5" s="27" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G5" s="32" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H5" s="30"/>
       <c r="I5" s="28" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="J5" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K5" s="49"/>
     </row>
@@ -1274,27 +1311,27 @@
         <v>5.2</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D6" s="27"/>
       <c r="E6" s="27" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F6" s="28" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H6" s="30"/>
       <c r="I6" s="28" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K6" s="49"/>
     </row>
@@ -1303,27 +1340,27 @@
         <v>5.2</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="27" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G7" s="29" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H7" s="33"/>
       <c r="I7" s="28" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="J7" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K7" s="49"/>
     </row>
@@ -1332,25 +1369,25 @@
         <v>5.2</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G8" s="30"/>
       <c r="H8" s="30"/>
       <c r="I8" s="28" t="s">
-        <v>72</v>
+        <v>35</v>
       </c>
       <c r="J8" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K8" s="49"/>
     </row>
@@ -1359,23 +1396,23 @@
         <v>5.2</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G9" s="30"/>
       <c r="H9" s="30"/>
       <c r="I9" s="28"/>
       <c r="J9" s="31" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K9" s="49"/>
     </row>
@@ -1384,25 +1421,25 @@
         <v>5.2</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="D10" s="27"/>
       <c r="E10" s="34" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F10" s="35" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="H10" s="36"/>
       <c r="I10" s="36"/>
       <c r="J10" s="31" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K10" s="49"/>
     </row>
@@ -1411,25 +1448,25 @@
         <v>5.2</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="34" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G11" s="36"/>
       <c r="H11" s="36"/>
       <c r="I11" s="37" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="J11" s="31" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K11" s="49"/>
     </row>
@@ -1438,27 +1475,27 @@
         <v>5.2</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="34" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G12" s="36" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H12" s="38"/>
       <c r="I12" s="37" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J12" s="31" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K12" s="49"/>
     </row>
@@ -1467,25 +1504,25 @@
         <v>5.2</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="34" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F13" s="37" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="H13" s="38"/>
       <c r="I13" s="37"/>
       <c r="J13" s="31" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K13" s="49"/>
     </row>
@@ -1494,23 +1531,23 @@
         <v>5.2</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>104</v>
+        <v>12</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D14" s="27"/>
       <c r="E14" s="34" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G14" s="36"/>
       <c r="H14" s="38"/>
       <c r="I14" s="37"/>
       <c r="J14" s="31" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K14" s="50"/>
     </row>
@@ -1519,30 +1556,30 @@
         <v>5.2</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="D15" s="13"/>
       <c r="E15" s="13" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H15" s="16"/>
       <c r="I15" s="14" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="J15" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K15" s="51" t="s">
-        <v>108</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -1550,27 +1587,27 @@
         <v>5.2</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="D16" s="13"/>
       <c r="E16" s="13" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H16" s="16"/>
       <c r="I16" s="14" t="s">
-        <v>71</v>
+        <v>24</v>
       </c>
       <c r="J16" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K16" s="52"/>
     </row>
@@ -1579,27 +1616,27 @@
         <v>5.2</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="D17" s="13"/>
       <c r="E17" s="13" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H17" s="16"/>
       <c r="I17" s="14" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J17" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K17" s="52"/>
     </row>
@@ -1608,25 +1645,25 @@
         <v>5.2</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="D18" s="13"/>
       <c r="E18" s="13" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="14"/>
       <c r="J18" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K18" s="52"/>
     </row>
@@ -1635,25 +1672,25 @@
         <v>5.2</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
       <c r="I19" s="14" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="J19" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K19" s="52"/>
     </row>
@@ -1662,53 +1699,53 @@
         <v>5.2</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G20" s="16"/>
       <c r="H20" s="16"/>
       <c r="I20" s="14"/>
       <c r="J20" s="17" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K20" s="53"/>
     </row>
-    <row r="21" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>5.2</v>
       </c>
-      <c r="B21" s="12" t="s">
-        <v>105</v>
+      <c r="B21" s="54" t="s">
+        <v>131</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="20" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>29</v>
+        <v>40</v>
+      </c>
+      <c r="G21" s="55" t="s">
+        <v>132</v>
       </c>
       <c r="H21" s="22"/>
       <c r="I21" s="22"/>
       <c r="J21" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="K21" s="51" t="s">
-        <v>109</v>
+        <v>42</v>
+      </c>
+      <c r="K21" s="56" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -1716,54 +1753,56 @@
         <v>5.2</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="20" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G22" s="22"/>
       <c r="H22" s="22"/>
       <c r="I22" s="23" t="s">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="J22" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="K22" s="52"/>
+        <v>42</v>
+      </c>
+      <c r="K22" s="52" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="23" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>5.2</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="20" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H23" s="24"/>
       <c r="I23" s="23" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="J23" s="17" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K23" s="52"/>
     </row>
@@ -1772,25 +1811,25 @@
         <v>5.2</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="20" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="H24" s="24"/>
       <c r="I24" s="23"/>
       <c r="J24" s="17" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K24" s="52"/>
     </row>
@@ -1799,23 +1838,23 @@
         <v>5.2</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="20" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G25" s="22"/>
       <c r="H25" s="24"/>
       <c r="I25" s="23"/>
       <c r="J25" s="17" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="K25" s="53"/>
     </row>
@@ -1824,27 +1863,27 @@
         <v>5.2</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="C26" s="7">
         <v>763264000</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>117</v>
+        <v>74</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>128</v>
+        <v>75</v>
       </c>
       <c r="H26" s="8"/>
       <c r="I26" s="8"/>
       <c r="J26" s="6" t="s">
-        <v>45</v>
+        <v>76</v>
       </c>
       <c r="K26" s="6"/>
     </row>
@@ -1853,28 +1892,28 @@
         <v>5.2</v>
       </c>
       <c r="B27" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="D27" s="11"/>
       <c r="E27" s="11" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="F27" s="40" t="s">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="G27" s="41"/>
       <c r="H27" s="10" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="I27" s="42"/>
       <c r="J27" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K27" s="45" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -1882,28 +1921,28 @@
         <v>5.2</v>
       </c>
       <c r="B28" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D28" s="46"/>
       <c r="E28" s="11" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="F28" s="43" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="G28" s="41"/>
       <c r="H28" s="10" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="I28" s="42"/>
       <c r="J28" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K28" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="31" x14ac:dyDescent="0.35">
@@ -1911,28 +1950,28 @@
         <v>5.2</v>
       </c>
       <c r="B29" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="D29" s="46"/>
       <c r="E29" s="11" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="F29" s="43" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="G29" s="41"/>
       <c r="H29" s="10" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="I29" s="42"/>
       <c r="J29" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K29" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
@@ -1940,28 +1979,28 @@
         <v>5.2</v>
       </c>
       <c r="B30" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="D30" s="46"/>
       <c r="E30" s="11" t="s">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="F30" s="40" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="G30" s="41"/>
       <c r="H30" s="10" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I30" s="42"/>
       <c r="J30" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K30" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
@@ -1969,28 +2008,28 @@
         <v>5.2</v>
       </c>
       <c r="B31" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>53</v>
+        <v>94</v>
       </c>
       <c r="D31" s="46"/>
       <c r="E31" s="11" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="F31" s="40" t="s">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="G31" s="41"/>
       <c r="H31" s="10" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I31" s="42"/>
       <c r="J31" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K31" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
@@ -1998,28 +2037,28 @@
         <v>5.2</v>
       </c>
       <c r="B32" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="D32" s="46"/>
       <c r="E32" s="11" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="F32" s="40" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="G32" s="41"/>
       <c r="H32" s="10" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="I32" s="42"/>
       <c r="J32" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K32" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2027,28 +2066,28 @@
         <v>5.2</v>
       </c>
       <c r="B33" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="D33" s="46"/>
       <c r="E33" s="11" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="G33" s="41"/>
       <c r="H33" s="10" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="I33" s="42"/>
       <c r="J33" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K33" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
@@ -2056,28 +2095,28 @@
         <v>5.2</v>
       </c>
       <c r="B34" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="D34" s="46"/>
       <c r="E34" s="11" t="s">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="F34" s="40" t="s">
-        <v>62</v>
+        <v>106</v>
       </c>
       <c r="G34" s="41"/>
       <c r="H34" s="10" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="I34" s="42"/>
       <c r="J34" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K34" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
@@ -2085,32 +2124,32 @@
         <v>5.2</v>
       </c>
       <c r="B35" s="43" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>63</v>
+        <v>107</v>
       </c>
       <c r="D35" s="46"/>
       <c r="E35" s="11" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="F35" s="40" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="G35" s="41" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I35" s="42" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="J35" s="41" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="K35" s="44" t="s">
-        <v>124</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
@@ -2118,10 +2157,10 @@
         <v>5.2</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="D36" s="12"/>
       <c r="E36" s="12"/>
@@ -2131,7 +2170,7 @@
       <c r="I36" s="12"/>
       <c r="J36" s="12"/>
       <c r="K36" s="12" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
@@ -2139,10 +2178,10 @@
         <v>5.2</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="D37" s="12"/>
       <c r="E37" s="12"/>
@@ -2152,7 +2191,7 @@
       <c r="I37" s="12"/>
       <c r="J37" s="12"/>
       <c r="K37" s="12" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
@@ -2160,10 +2199,10 @@
         <v>5.2</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>68</v>
+        <v>118</v>
       </c>
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
@@ -2173,7 +2212,7 @@
       <c r="I38" s="12"/>
       <c r="J38" s="12"/>
       <c r="K38" s="12" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
@@ -2181,10 +2220,10 @@
         <v>5.2</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="D39" s="12"/>
       <c r="E39" s="12"/>
@@ -2194,7 +2233,7 @@
       <c r="I39" s="12"/>
       <c r="J39" s="12"/>
       <c r="K39" s="12" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
@@ -2202,10 +2241,10 @@
         <v>5.2</v>
       </c>
       <c r="B40" s="26" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C40" s="27" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D40" s="26"/>
       <c r="E40" s="26"/>
@@ -2221,10 +2260,10 @@
         <v>5.2</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D41" s="26"/>
       <c r="E41" s="26"/>
@@ -2240,10 +2279,10 @@
         <v>5.2</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D42" s="26"/>
       <c r="E42" s="26"/>
@@ -2256,24 +2295,24 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B44" s="5" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B45" s="9" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B46" s="39" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="K4:K14"/>
     <mergeCell ref="K15:K20"/>
-    <mergeCell ref="K21:K25"/>
+    <mergeCell ref="K22:K25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G4" r:id="rId1" xr:uid="{F1EC2680-9018-4C74-B22B-CD92FC568C41}"/>

</xml_diff>

<commit_message>
Add changes to IDN07, PAT10, TRA70, CAP01
IDN07 - UKRR_UID for all patients
PAT10 - NHSBT_NO re-instituted
TRA70 - UKTR_ID removed
CAP01 - Date of assessment start
CAP04 - Date of assessment end
</commit_message>
<xml_diff>
--- a/Excel/v5/UKRR DataSet Amendments.xlsx
+++ b/Excel/v5/UKRR DataSet Amendments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marta.badji\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9AFD743-246A-4E6D-BC78-CF07D4AE2520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6DAA98-A7E1-4D59-B308-8B0EB5A8A071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Amendments" sheetId="21" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="160">
   <si>
     <t>Amendments</t>
   </si>
@@ -455,6 +455,72 @@
   <si>
     <t>This item replaces DXS07.
 Codes updated from the V5 values (N, TYPE1, TYPE2, TYPE UNKNOWN) to codelist RR52. 'TYPE I' and 'TYPE II' restored to match the V4 codes, correcting the typo introduced in V5 as 'TYPE1' and 'TYPE2'.</t>
+  </si>
+  <si>
+    <t>IDN07</t>
+  </si>
+  <si>
+    <t>C20</t>
+  </si>
+  <si>
+    <t>Unique identifier not attributable to patient.</t>
+  </si>
+  <si>
+    <t>Site code plus internal record number or similar eg. REE01-12345</t>
+  </si>
+  <si>
+    <t>Patient/PatientNumber</t>
+  </si>
+  <si>
+    <t>Removed IF/Qualification, made item mandatory for all patients</t>
+  </si>
+  <si>
+    <t>PAT10</t>
+  </si>
+  <si>
+    <t>N6</t>
+  </si>
+  <si>
+    <t>NHSBT number</t>
+  </si>
+  <si>
+    <t>Reinstated from v4.2, replaces TRA70.</t>
+  </si>
+  <si>
+    <t>TRA70</t>
+  </si>
+  <si>
+    <t>NHSBT Field ID: UKTR_ID</t>
+  </si>
+  <si>
+    <t>UKTR recipient ID</t>
+  </si>
+  <si>
+    <t>Numeric field up to 6 digits</t>
+  </si>
+  <si>
+    <t>Procedures/Transplant</t>
+  </si>
+  <si>
+    <t>Replaced by PAT10.</t>
+  </si>
+  <si>
+    <t>CAP01</t>
+  </si>
+  <si>
+    <t>Date of assessment start</t>
+  </si>
+  <si>
+    <t>Assesments</t>
+  </si>
+  <si>
+    <t>Date of assessment changed to Date of assessment start</t>
+  </si>
+  <si>
+    <t>CAP04</t>
+  </si>
+  <si>
+    <t>Date of assessment end</t>
   </si>
 </sst>
 </file>
@@ -662,7 +728,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -805,6 +871,56 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1199,7 +1315,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17.08203125" customWidth="1"/>
@@ -1255,96 +1371,94 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>5.2</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="46" t="s">
+        <v>139</v>
+      </c>
+      <c r="F4" s="57" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" s="10"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="58" t="s">
+        <v>142</v>
+      </c>
+      <c r="K4" s="58" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>5.2</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="60" t="s">
+        <v>145</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="G5" s="61"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="K5" s="23" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5.2</v>
+      </c>
+      <c r="B6" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="29" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="30"/>
-      <c r="I4" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="51" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="31" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>5.2</v>
-      </c>
-      <c r="B5" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="30"/>
-      <c r="I5" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="52"/>
-    </row>
-    <row r="6" spans="1:11" ht="155" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>5.2</v>
-      </c>
-      <c r="B6" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="30"/>
-      <c r="I6" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="52"/>
-    </row>
-    <row r="7" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="65" t="s">
+        <v>148</v>
+      </c>
+      <c r="D6" s="66" t="s">
+        <v>149</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="F6" s="67" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="68" t="s">
+        <v>151</v>
+      </c>
+      <c r="H6" s="69"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="K6" s="37" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5.2</v>
       </c>
@@ -1352,28 +1466,30 @@
         <v>12</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="D7" s="27"/>
       <c r="E7" s="27" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G7" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="33"/>
+      <c r="H7" s="30"/>
       <c r="I7" s="28" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="J7" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="K7" s="52"/>
-    </row>
-    <row r="8" spans="1:11" ht="93" x14ac:dyDescent="0.35">
+      <c r="K7" s="51" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5.2</v>
       </c>
@@ -1381,26 +1497,28 @@
         <v>12</v>
       </c>
       <c r="C8" s="27" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D8" s="27"/>
       <c r="E8" s="27" t="s">
         <v>21</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="30"/>
+        <v>22</v>
+      </c>
+      <c r="G8" s="32" t="s">
+        <v>23</v>
+      </c>
       <c r="H8" s="30"/>
       <c r="I8" s="28" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="J8" s="31" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="52"/>
     </row>
-    <row r="9" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="155" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>5.2</v>
       </c>
@@ -1408,18 +1526,22 @@
         <v>12</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" s="30"/>
+        <v>27</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>28</v>
+      </c>
       <c r="H9" s="30"/>
-      <c r="I9" s="28"/>
+      <c r="I9" s="28" t="s">
+        <v>29</v>
+      </c>
       <c r="J9" s="31" t="s">
         <v>18</v>
       </c>
@@ -1433,26 +1555,28 @@
         <v>12</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D10" s="27"/>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="H10" s="36"/>
-      <c r="I10" s="36"/>
+      <c r="F10" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="33"/>
+      <c r="I10" s="28" t="s">
+        <v>32</v>
+      </c>
       <c r="J10" s="31" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="K10" s="52"/>
     </row>
-    <row r="11" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="93" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>5.2</v>
       </c>
@@ -1460,26 +1584,26 @@
         <v>12</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D11" s="27"/>
-      <c r="E11" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="37" t="s">
-        <v>45</v>
+      <c r="E11" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="28" t="s">
+        <v>35</v>
       </c>
       <c r="J11" s="31" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="K11" s="52"/>
     </row>
-    <row r="12" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>5.2</v>
       </c>
@@ -1487,24 +1611,20 @@
         <v>12</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D12" s="27"/>
-      <c r="E12" s="34" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" s="36" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="38"/>
-      <c r="I12" s="37" t="s">
-        <v>48</v>
-      </c>
+      <c r="E12" s="27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="28"/>
       <c r="J12" s="31" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="K12" s="52"/>
     </row>
@@ -1516,26 +1636,26 @@
         <v>12</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="G13" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H13" s="38"/>
-      <c r="I13" s="37"/>
+      <c r="F13" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
       <c r="J13" s="31" t="s">
         <v>42</v>
       </c>
       <c r="K13" s="52"/>
     </row>
-    <row r="14" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>5.2</v>
       </c>
@@ -1543,113 +1663,107 @@
         <v>12</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D14" s="27"/>
       <c r="E14" s="34" t="s">
         <v>37</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G14" s="36"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="37"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="37" t="s">
+        <v>45</v>
+      </c>
       <c r="J14" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="K14" s="53"/>
-    </row>
-    <row r="15" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="K14" s="52"/>
+    </row>
+    <row r="15" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>5.2</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="H15" s="16"/>
-      <c r="I15" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="J15" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="K15" s="54" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="B15" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="27"/>
+      <c r="E15" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="G15" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="38"/>
+      <c r="I15" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" s="52"/>
+    </row>
+    <row r="16" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>5.2</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="16"/>
-      <c r="I16" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="J16" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="K16" s="55"/>
-    </row>
-    <row r="17" spans="1:11" ht="155" x14ac:dyDescent="0.35">
+      <c r="B16" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="27"/>
+      <c r="E16" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="H16" s="38"/>
+      <c r="I16" s="37"/>
+      <c r="J16" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="52"/>
+    </row>
+    <row r="17" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>5.2</v>
       </c>
-      <c r="B17" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="16"/>
-      <c r="I17" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="J17" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="K17" s="55"/>
-    </row>
-    <row r="18" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D17" s="27"/>
+      <c r="E17" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="36"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="37"/>
+      <c r="J17" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="K17" s="53"/>
+    </row>
+    <row r="18" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>5.2</v>
       </c>
@@ -1657,53 +1771,59 @@
         <v>54</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D18" s="13"/>
       <c r="E18" s="13" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G18" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H18" s="19"/>
-      <c r="I18" s="14"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="14" t="s">
+        <v>56</v>
+      </c>
       <c r="J18" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="K18" s="55"/>
-    </row>
-    <row r="19" spans="1:11" ht="77.5" x14ac:dyDescent="0.35">
+      <c r="K18" s="54" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>5.2</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="G19" s="16"/>
+        <v>22</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>23</v>
+      </c>
       <c r="H19" s="16"/>
       <c r="I19" s="14" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="J19" s="17" t="s">
         <v>18</v>
       </c>
       <c r="K19" s="55"/>
     </row>
-    <row r="20" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" ht="155" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>5.2</v>
       </c>
@@ -1711,53 +1831,55 @@
         <v>58</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="13" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="G20" s="16"/>
+        <v>27</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>28</v>
+      </c>
       <c r="H20" s="16"/>
-      <c r="I20" s="14"/>
+      <c r="I20" s="14" t="s">
+        <v>29</v>
+      </c>
       <c r="J20" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="K20" s="56"/>
-    </row>
-    <row r="21" spans="1:11" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K20" s="55"/>
+    </row>
+    <row r="21" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>5.2</v>
       </c>
-      <c r="B21" s="48" t="s">
-        <v>131</v>
+      <c r="B21" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D21" s="13"/>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="G21" s="49" t="s">
-        <v>136</v>
-      </c>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
+      <c r="F21" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="19"/>
+      <c r="I21" s="14"/>
       <c r="J21" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="K21" s="50" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="K21" s="55"/>
+    </row>
+    <row r="22" spans="1:11" ht="77.5" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>5.2</v>
       </c>
@@ -1765,84 +1887,80 @@
         <v>54</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D22" s="13"/>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="J22" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="55"/>
+    </row>
+    <row r="23" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>5.2</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F22" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="J22" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="K22" s="55" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>5.2</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="D23" s="13"/>
-      <c r="E23" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="G23" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="H23" s="24"/>
-      <c r="I23" s="23" t="s">
-        <v>69</v>
-      </c>
+      <c r="F23" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="I23" s="14"/>
       <c r="J23" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="K23" s="55"/>
-    </row>
-    <row r="24" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="K23" s="56"/>
+    </row>
+    <row r="24" spans="1:11" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>5.2</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>54</v>
+      <c r="B24" s="48" t="s">
+        <v>131</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D24" s="13"/>
       <c r="E24" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="H24" s="24"/>
-      <c r="I24" s="23"/>
+      <c r="F24" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="G24" s="49" t="s">
+        <v>136</v>
+      </c>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
       <c r="J24" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="K24" s="55"/>
-    </row>
-    <row r="25" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K24" s="50" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>5.2</v>
       </c>
@@ -1850,140 +1968,138 @@
         <v>54</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="20" t="s">
         <v>37</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G25" s="22"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="23"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23" t="s">
+        <v>67</v>
+      </c>
       <c r="J25" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="K25" s="56"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K25" s="55" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>5.2</v>
       </c>
       <c r="B26" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="13"/>
+      <c r="E26" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="G26" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="24"/>
+      <c r="I26" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="K26" s="55"/>
+    </row>
+    <row r="27" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>5.2</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H27" s="24"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="K27" s="55"/>
+    </row>
+    <row r="28" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>5.2</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" s="22"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="K28" s="56"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>5.2</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="7">
+      <c r="C29" s="7">
         <v>763264000</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D29" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="E29" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F29" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="G26" s="8" t="s">
+      <c r="G29" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="6" t="s">
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="K26" s="6"/>
-    </row>
-    <row r="27" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>5.2</v>
-      </c>
-      <c r="B27" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F27" s="40" t="s">
-        <v>79</v>
-      </c>
-      <c r="G27" s="41"/>
-      <c r="H27" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I27" s="42"/>
-      <c r="J27" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="K27" s="45" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" ht="31" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>5.2</v>
-      </c>
-      <c r="B28" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D28" s="46"/>
-      <c r="E28" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="F28" s="43" t="s">
-        <v>85</v>
-      </c>
-      <c r="G28" s="41"/>
-      <c r="H28" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="I28" s="42"/>
-      <c r="J28" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="K28" s="44" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="31" x14ac:dyDescent="0.35">
-      <c r="A29">
-        <v>5.2</v>
-      </c>
-      <c r="B29" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="D29" s="46"/>
-      <c r="E29" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="F29" s="43" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="41"/>
-      <c r="H29" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="I29" s="42"/>
-      <c r="J29" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="K29" s="44" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K29" s="6"/>
+    </row>
+    <row r="30" spans="1:11" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>5.2</v>
       </c>
@@ -1991,28 +2107,28 @@
         <v>130</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="46"/>
+        <v>77</v>
+      </c>
+      <c r="D30" s="11"/>
       <c r="E30" s="11" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="F30" s="40" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="G30" s="41"/>
       <c r="H30" s="10" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="I30" s="42"/>
       <c r="J30" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="K30" s="44" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="K30" s="45" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>5.2</v>
       </c>
@@ -2020,18 +2136,18 @@
         <v>130</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="D31" s="46"/>
       <c r="E31" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="F31" s="40" t="s">
-        <v>95</v>
+      <c r="F31" s="43" t="s">
+        <v>85</v>
       </c>
       <c r="G31" s="41"/>
       <c r="H31" s="10" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="I31" s="42"/>
       <c r="J31" s="41" t="s">
@@ -2041,7 +2157,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>5.2</v>
       </c>
@@ -2049,18 +2165,18 @@
         <v>130</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D32" s="46"/>
       <c r="E32" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="F32" s="40" t="s">
-        <v>98</v>
+        <v>84</v>
+      </c>
+      <c r="F32" s="43" t="s">
+        <v>89</v>
       </c>
       <c r="G32" s="41"/>
       <c r="H32" s="10" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="I32" s="42"/>
       <c r="J32" s="41" t="s">
@@ -2078,18 +2194,18 @@
         <v>130</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D33" s="46"/>
       <c r="E33" s="11" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F33" s="40" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="G33" s="41"/>
       <c r="H33" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="I33" s="42"/>
       <c r="J33" s="41" t="s">
@@ -2107,18 +2223,18 @@
         <v>130</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D34" s="46"/>
       <c r="E34" s="11" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="F34" s="40" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="G34" s="41"/>
       <c r="H34" s="10" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="I34" s="42"/>
       <c r="J34" s="41" t="s">
@@ -2136,24 +2252,20 @@
         <v>130</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="D35" s="46"/>
       <c r="E35" s="11" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="F35" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="G35" s="41" t="s">
-        <v>110</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="G35" s="41"/>
       <c r="H35" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="I35" s="42" t="s">
-        <v>112</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="I35" s="42"/>
       <c r="J35" s="41" t="s">
         <v>81</v>
       </c>
@@ -2165,190 +2277,333 @@
       <c r="A36">
         <v>5.2</v>
       </c>
-      <c r="B36" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12" t="s">
-        <v>115</v>
+      <c r="B36" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="46"/>
+      <c r="E36" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="F36" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="G36" s="41"/>
+      <c r="H36" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I36" s="42"/>
+      <c r="J36" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="K36" s="44" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>5.2</v>
       </c>
-      <c r="B37" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12" t="s">
-        <v>117</v>
+      <c r="B37" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" s="46"/>
+      <c r="E37" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="F37" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="G37" s="41"/>
+      <c r="H37" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I37" s="42"/>
+      <c r="J37" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="K37" s="44" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>5.2</v>
       </c>
-      <c r="B38" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B38" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="46"/>
+      <c r="E38" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F38" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="G38" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="I38" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="J38" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="K38" s="44" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="31" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>5.2</v>
       </c>
-      <c r="B39" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="12"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="B39" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D39" s="71"/>
+      <c r="E39" s="72" t="s">
+        <v>37</v>
+      </c>
+      <c r="F39" s="46" t="s">
+        <v>155</v>
+      </c>
+      <c r="G39" s="40"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="42" t="s">
+        <v>156</v>
+      </c>
+      <c r="K39" s="58" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>5.2</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>135</v>
+        <v>58</v>
+      </c>
+      <c r="C40" s="73" t="s">
+        <v>158</v>
       </c>
       <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="12"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="48" t="s">
-        <v>134</v>
-      </c>
+      <c r="E40" s="74" t="s">
+        <v>37</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G40" s="61"/>
+      <c r="H40" s="62"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="K40" s="23"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>5.2</v>
       </c>
-      <c r="B41" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="26"/>
-      <c r="K41" s="26"/>
+      <c r="B41" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D41" s="12"/>
+      <c r="E41" s="12"/>
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>5.2</v>
       </c>
-      <c r="B42" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="C42" s="27" t="s">
-        <v>125</v>
-      </c>
-      <c r="D42" s="26"/>
-      <c r="E42" s="26"/>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="26"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="26"/>
-      <c r="K42" s="26"/>
+      <c r="B42" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D42" s="12"/>
+      <c r="E42" s="12"/>
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>5.2</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="12"/>
+      <c r="E43" s="12"/>
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>5.2</v>
+      </c>
+      <c r="B44" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="12"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>5.2</v>
+      </c>
+      <c r="B45" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="48" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>5.2</v>
+      </c>
+      <c r="B46" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="26"/>
+      <c r="I46" s="26"/>
+      <c r="J46" s="26"/>
+      <c r="K46" s="26"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>5.2</v>
+      </c>
+      <c r="B47" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="C43" s="27" t="s">
+      <c r="C47" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="D47" s="26"/>
+      <c r="E47" s="26"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="26"/>
+      <c r="I47" s="26"/>
+      <c r="J47" s="26"/>
+      <c r="K47" s="26"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>5.2</v>
+      </c>
+      <c r="B48" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="D43" s="26"/>
-      <c r="E43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="26"/>
-      <c r="J43" s="26"/>
-      <c r="K43" s="26"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B45" s="5" t="s">
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
+      <c r="H48" s="26"/>
+      <c r="I48" s="26"/>
+      <c r="J48" s="26"/>
+      <c r="K48" s="26"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B50" s="5" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B46" s="9" t="s">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B51" s="9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B47" s="39" t="s">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B52" s="39" t="s">
         <v>129</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="K4:K14"/>
-    <mergeCell ref="K15:K20"/>
-    <mergeCell ref="K22:K25"/>
+    <mergeCell ref="K7:K17"/>
+    <mergeCell ref="K18:K23"/>
+    <mergeCell ref="K25:K28"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G4" r:id="rId1" xr:uid="{F1EC2680-9018-4C74-B22B-CD92FC568C41}"/>
-    <hyperlink ref="G7" r:id="rId2" xr:uid="{40922429-9AB4-4D19-85B5-192B08239677}"/>
-    <hyperlink ref="G15" r:id="rId3" xr:uid="{203FFA4B-5962-487D-8C1A-FB7E40FB3065}"/>
-    <hyperlink ref="G18" r:id="rId4" xr:uid="{5CC3261D-6C9B-4396-8FB1-1D69B57AF4A2}"/>
+    <hyperlink ref="G7" r:id="rId1" xr:uid="{F1EC2680-9018-4C74-B22B-CD92FC568C41}"/>
+    <hyperlink ref="G10" r:id="rId2" xr:uid="{40922429-9AB4-4D19-85B5-192B08239677}"/>
+    <hyperlink ref="G18" r:id="rId3" xr:uid="{203FFA4B-5962-487D-8C1A-FB7E40FB3065}"/>
+    <hyperlink ref="G21" r:id="rId4" xr:uid="{5CC3261D-6C9B-4396-8FB1-1D69B57AF4A2}"/>
   </hyperlinks>
   <pageMargins left="0.70833333333333304" right="0.70833333333333304" top="0.74791666666666701" bottom="0.74861111111111101" header="0.511811023622047" footer="0.31527777777777799"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId5"/>

</xml_diff>